<commit_message>
feat: Implement application settings dialog for theme and default rent management
- Added SettingsController to manage application settings.
- Created a settings dialog to allow users to manage theme and default rent settings.
- Integrated theme application across main window and various tabs.
- Enhanced payment dialog to support custom payment types and persist them in settings.
- Updated rent dashboard and management tabs to apply themes dynamically.
- Improved layout and styling for better user experience in rent management.
- Added functionality to handle late fees and notifications for upcoming due dates.
- Fixed bugs related to dark mode visibility and settings changes.
- Updated documentation and logging for better clarity and maintenance.
</commit_message>
<xml_diff>
--- a/Financial Manager/resources/Maria(Current)_rent_export.xlsx
+++ b/Financial Manager/resources/Maria(Current)_rent_export.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Main" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2026" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Main'!$A$1:$H$71</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'2026'!$A$1:$H$34</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Main'!$A$1:$H$74</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'2026'!$A$1:$H$37</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'2025'!$A$1:$H$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -671,7 +671,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Report Generated: 2026-03-08 12:33:14</t>
+          <t>Report Generated: 2026-04-02 23:23:07</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>March 2026</t>
+          <t>April 2026</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>1750</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="20">
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>1750</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="24">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="H50" s="12" t="inlineStr">
         <is>
-          <t>2 payments of 500 $ targetted to pay off random delinquent months</t>
+          <t>2 payments of 500 $ targeted to pay off random delinquent months</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="C57" s="21" t="inlineStr">
         <is>
-          <t>Overpayment Credit (Applied: $350.00)</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="D57" s="21" t="inlineStr">
@@ -1919,7 +1919,7 @@
       <c r="G57" s="20" t="inlineStr"/>
       <c r="H57" s="21" t="inlineStr">
         <is>
-          <t>RANDOM TARGETTED MONTH TO PAY OFF</t>
+          <t>RANDOM TARGETED MONTH TO PAY OFF</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="C59" s="21" t="inlineStr">
         <is>
-          <t>Overpayment Credit (Applied: $450.00)</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="D59" s="21" t="inlineStr">
@@ -1974,18 +1974,18 @@
       </c>
       <c r="E59" s="21" t="inlineStr">
         <is>
-          <t>Partial Payment</t>
+          <t>Overpayment</t>
         </is>
       </c>
       <c r="F59" s="21" t="inlineStr">
         <is>
-          <t>$400.00 remaining</t>
+          <t>Overpaid by $200.00</t>
         </is>
       </c>
       <c r="G59" s="20" t="inlineStr"/>
       <c r="H59" s="21" t="inlineStr">
         <is>
-          <t>RANDOM TARGETTED MONTH TO APPLY OVERCREDIT</t>
+          <t>RANDOM TARGETED MONTH TO APPLY OVERCREDIT</t>
         </is>
       </c>
     </row>
@@ -2006,146 +2006,179 @@
           <t>2026-02</t>
         </is>
       </c>
-      <c r="E60" s="23" t="inlineStr">
-        <is>
-          <t>Partial Payment</t>
-        </is>
-      </c>
-      <c r="F60" s="24" t="inlineStr">
-        <is>
-          <t>$400.00 remaining</t>
+      <c r="E60" s="22" t="inlineStr">
+        <is>
+          <t>Overpayment</t>
+        </is>
+      </c>
+      <c r="F60" s="22" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00</t>
         </is>
       </c>
       <c r="G60" s="11" t="inlineStr"/>
       <c r="H60" s="12" t="inlineStr"/>
     </row>
+    <row r="61">
+      <c r="A61" s="10" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B61" s="11" t="n">
+        <v>600</v>
+      </c>
+      <c r="C61" s="12" t="inlineStr">
+        <is>
+          <t>Zelle</t>
+        </is>
+      </c>
+      <c r="D61" s="17" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="E61" s="22" t="inlineStr">
+        <is>
+          <t>Overpayment</t>
+        </is>
+      </c>
+      <c r="F61" s="22" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00</t>
+        </is>
+      </c>
+      <c r="G61" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="H61" s="12" t="inlineStr"/>
+    </row>
     <row r="62">
-      <c r="A62" s="3" t="inlineStr">
+      <c r="A62" s="10" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B62" s="11" t="n">
+        <v>650</v>
+      </c>
+      <c r="C62" s="12" t="inlineStr">
+        <is>
+          <t>Zelle</t>
+        </is>
+      </c>
+      <c r="D62" s="18" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="E62" s="23" t="inlineStr">
+        <is>
+          <t>Partial Payment</t>
+        </is>
+      </c>
+      <c r="F62" s="24" t="inlineStr">
+        <is>
+          <t>$500.00 remaining</t>
+        </is>
+      </c>
+      <c r="G62" s="11" t="inlineStr"/>
+      <c r="H62" s="12" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="19" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B63" s="20" t="n">
+        <v>200</v>
+      </c>
+      <c r="C63" s="21" t="inlineStr">
+        <is>
+          <t>Overpayment Credit (Applied: $200.00)</t>
+        </is>
+      </c>
+      <c r="D63" s="21" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="E63" s="21" t="inlineStr">
+        <is>
+          <t>Partial Payment</t>
+        </is>
+      </c>
+      <c r="F63" s="21" t="inlineStr">
+        <is>
+          <t>$500.00 remaining</t>
+        </is>
+      </c>
+      <c r="G63" s="20" t="inlineStr"/>
+      <c r="H63" s="21" t="inlineStr">
+        <is>
+          <t>Random applied to current month</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
         <is>
           <t>MONTHLY BALANCE SUMMARY (Filtered)</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="9" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="9" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B63" s="9" t="inlineStr">
+      <c r="B66" s="9" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C63" s="9" t="inlineStr">
+      <c r="C66" s="9" t="inlineStr">
         <is>
           <t>Rent Due</t>
         </is>
       </c>
-      <c r="D63" s="9" t="inlineStr">
+      <c r="D66" s="9" t="inlineStr">
         <is>
           <t>Total Paid</t>
         </is>
       </c>
-      <c r="E63" s="9" t="inlineStr">
+      <c r="E66" s="9" t="inlineStr">
         <is>
           <t>Balance</t>
         </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="25" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B64" s="26" t="inlineStr">
-        <is>
-          <t>Partial Payment</t>
-        </is>
-      </c>
-      <c r="C64" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D64" s="27" t="n">
-        <v>950</v>
-      </c>
-      <c r="E64" s="28" t="n">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="25" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B65" s="29" t="inlineStr">
-        <is>
-          <t>Not Paid</t>
-        </is>
-      </c>
-      <c r="C65" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D65" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E65" s="30" t="n">
-        <v>1350</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="25" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B66" s="31" t="inlineStr">
-        <is>
-          <t>Due Soon</t>
-        </is>
-      </c>
-      <c r="C66" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D66" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E66" s="32" t="n">
-        <v>1350</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="25" t="inlineStr">
         <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B67" s="33" t="inlineStr">
-        <is>
-          <t>Not Due</t>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B67" s="26" t="inlineStr">
+        <is>
+          <t>Partial Payment</t>
         </is>
       </c>
       <c r="C67" s="27" t="n">
         <v>1350</v>
       </c>
       <c r="D67" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E67" s="34" t="n">
-        <v>0</v>
+        <v>850</v>
+      </c>
+      <c r="E67" s="28" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="25" t="inlineStr">
         <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B68" s="33" t="inlineStr">
-        <is>
-          <t>Not Due</t>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B68" s="29" t="inlineStr">
+        <is>
+          <t>Not Paid</t>
         </is>
       </c>
       <c r="C68" s="27" t="n">
@@ -2154,19 +2187,19 @@
       <c r="D68" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="E68" s="34" t="n">
-        <v>0</v>
+      <c r="E68" s="30" t="n">
+        <v>1350</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="25" t="inlineStr">
         <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B69" s="33" t="inlineStr">
-        <is>
-          <t>Not Due</t>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B69" s="31" t="inlineStr">
+        <is>
+          <t>Due Soon</t>
         </is>
       </c>
       <c r="C69" s="27" t="n">
@@ -2175,14 +2208,14 @@
       <c r="D69" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="E69" s="34" t="n">
-        <v>0</v>
+      <c r="E69" s="32" t="n">
+        <v>1350</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="25" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B70" s="33" t="inlineStr">
@@ -2203,7 +2236,7 @@
     <row r="71">
       <c r="A71" s="25" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B71" s="33" t="inlineStr">
@@ -2218,13 +2251,76 @@
         <v>0</v>
       </c>
       <c r="E71" s="34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="25" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B72" s="33" t="inlineStr">
+        <is>
+          <t>Not Due</t>
+        </is>
+      </c>
+      <c r="C72" s="27" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D72" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="25" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B73" s="33" t="inlineStr">
+        <is>
+          <t>Not Due</t>
+        </is>
+      </c>
+      <c r="C73" s="27" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D73" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="25" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B74" s="33" t="inlineStr">
+        <is>
+          <t>Not Due</t>
+        </is>
+      </c>
+      <c r="C74" s="27" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D74" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="34" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A65:H65"/>
     <mergeCell ref="A24:H24"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A14:H14"/>
@@ -2242,7 +2338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2258,7 +2354,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Report Generated: 2026-03-08 12:33:14 | Year: 2026 (Filtered by Payment Month)</t>
+          <t>Report Generated: 2026-04-02 23:23:09 | Year: 2026 (Filtered by Payment Month)</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2508,7 @@
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>Overpayment Credit (Applied: $450.00)</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
@@ -2422,18 +2518,18 @@
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>Partial Payment</t>
+          <t>Overpayment</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
         <is>
-          <t>$400.00 remaining</t>
+          <t>Overpaid by $200.00</t>
         </is>
       </c>
       <c r="G13" s="20" t="inlineStr"/>
       <c r="H13" s="21" t="inlineStr">
         <is>
-          <t>RANDOM TARGETTED MONTH TO APPLY OVERCREDIT</t>
+          <t>RANDOM TARGETED MONTH TO APPLY OVERCREDIT</t>
         </is>
       </c>
     </row>
@@ -2454,225 +2550,258 @@
           <t>2026-02</t>
         </is>
       </c>
-      <c r="E14" s="23" t="inlineStr">
-        <is>
-          <t>Partial Payment</t>
-        </is>
-      </c>
-      <c r="F14" s="24" t="inlineStr">
-        <is>
-          <t>$400.00 remaining</t>
+      <c r="E14" s="22" t="inlineStr">
+        <is>
+          <t>Overpayment</t>
+        </is>
+      </c>
+      <c r="F14" s="22" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr"/>
       <c r="H14" s="12" t="inlineStr"/>
     </row>
+    <row r="15">
+      <c r="A15" s="10" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>600</v>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Zelle</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>Overpayment</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="H15" s="12" t="inlineStr"/>
+    </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="10" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>650</v>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Zelle</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="E16" s="23" t="inlineStr">
+        <is>
+          <t>Partial Payment</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>$500.00 remaining</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr"/>
+      <c r="H16" s="12" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B17" s="20" t="n">
+        <v>200</v>
+      </c>
+      <c r="C17" s="21" t="inlineStr">
+        <is>
+          <t>Overpayment Credit (Applied: $200.00)</t>
+        </is>
+      </c>
+      <c r="D17" s="21" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="E17" s="21" t="inlineStr">
+        <is>
+          <t>Partial Payment</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr">
+        <is>
+          <t>$500.00 remaining</t>
+        </is>
+      </c>
+      <c r="G17" s="20" t="inlineStr"/>
+      <c r="H17" s="21" t="inlineStr">
+        <is>
+          <t>Random applied to current month</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>YEAR SUMMARY - 2026 (Tax Purposes)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Total Actual Payments</t>
         </is>
       </c>
-      <c r="B17" s="35" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="B20" s="35" t="n">
+        <v>3250</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Total Rent Due</t>
         </is>
       </c>
-      <c r="B18" s="36" t="n">
+      <c r="B21" s="36" t="n">
         <v>16200</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Net Difference</t>
         </is>
       </c>
-      <c r="B19" s="37" t="n">
-        <v>-14200</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="B22" s="37" t="n">
+        <v>-12950</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>MONTHLY BALANCE SUMMARY - 2026</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>Rent Due</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>Total Paid</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t>Balance</t>
         </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="25" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B23" s="38" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="C23" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D23" s="27" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E23" s="39" t="n">
-        <v>-150</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="25" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B24" s="26" t="inlineStr">
-        <is>
-          <t>Partial Payment</t>
-        </is>
-      </c>
-      <c r="C24" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D24" s="27" t="n">
-        <v>950</v>
-      </c>
-      <c r="E24" s="28" t="n">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="25" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B25" s="29" t="inlineStr">
-        <is>
-          <t>Not Paid</t>
-        </is>
-      </c>
-      <c r="C25" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D25" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="30" t="n">
-        <v>1350</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="25" t="inlineStr">
         <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B26" s="31" t="inlineStr">
-        <is>
-          <t>Due Soon</t>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B26" s="38" t="inlineStr">
+        <is>
+          <t>Overpayment</t>
         </is>
       </c>
       <c r="C26" s="27" t="n">
         <v>1350</v>
       </c>
       <c r="D26" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="32" t="n">
-        <v>1350</v>
+        <v>1500</v>
+      </c>
+      <c r="E26" s="39" t="n">
+        <v>-150</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B27" s="33" t="inlineStr">
-        <is>
-          <t>Not Due</t>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B27" s="38" t="inlineStr">
+        <is>
+          <t>Overpayment</t>
         </is>
       </c>
       <c r="C27" s="27" t="n">
         <v>1350</v>
       </c>
       <c r="D27" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="34" t="n">
-        <v>0</v>
+        <v>1550</v>
+      </c>
+      <c r="E27" s="39" t="n">
+        <v>-200</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="25" t="inlineStr">
         <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B28" s="33" t="inlineStr">
-        <is>
-          <t>Not Due</t>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>Partial Payment</t>
         </is>
       </c>
       <c r="C28" s="27" t="n">
         <v>1350</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="34" t="n">
-        <v>0</v>
+        <v>850</v>
+      </c>
+      <c r="E28" s="28" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="25" t="inlineStr">
         <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B29" s="33" t="inlineStr">
-        <is>
-          <t>Not Due</t>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B29" s="29" t="inlineStr">
+        <is>
+          <t>Not Paid</t>
         </is>
       </c>
       <c r="C29" s="27" t="n">
@@ -2681,19 +2810,19 @@
       <c r="D29" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="E29" s="34" t="n">
-        <v>0</v>
+      <c r="E29" s="30" t="n">
+        <v>1350</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="25" t="inlineStr">
         <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B30" s="33" t="inlineStr">
-        <is>
-          <t>Not Due</t>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="inlineStr">
+        <is>
+          <t>Due Soon</t>
         </is>
       </c>
       <c r="C30" s="27" t="n">
@@ -2702,14 +2831,14 @@
       <c r="D30" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="E30" s="34" t="n">
-        <v>0</v>
+      <c r="E30" s="32" t="n">
+        <v>1350</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="25" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B31" s="33" t="inlineStr">
@@ -2730,7 +2859,7 @@
     <row r="32">
       <c r="A32" s="25" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B32" s="33" t="inlineStr">
@@ -2751,7 +2880,7 @@
     <row r="33">
       <c r="A33" s="25" t="inlineStr">
         <is>
-          <t>2026-11</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B33" s="33" t="inlineStr">
@@ -2772,7 +2901,7 @@
     <row r="34">
       <c r="A34" s="25" t="inlineStr">
         <is>
-          <t>2026-12</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="B34" s="33" t="inlineStr">
@@ -2787,16 +2916,79 @@
         <v>0</v>
       </c>
       <c r="E34" s="34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="25" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B35" s="33" t="inlineStr">
+        <is>
+          <t>Not Due</t>
+        </is>
+      </c>
+      <c r="C35" s="27" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D35" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="25" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B36" s="33" t="inlineStr">
+        <is>
+          <t>Not Due</t>
+        </is>
+      </c>
+      <c r="C36" s="27" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D36" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="25" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B37" s="33" t="inlineStr">
+        <is>
+          <t>Not Due</t>
+        </is>
+      </c>
+      <c r="C37" s="27" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D37" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="34" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A24:H24"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
@@ -2827,7 +3019,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Report Generated: 2026-03-08 12:33:15 | Year: 2025 (Filtered by Date Received)</t>
+          <t>Report Generated: 2026-04-02 23:23:10 | Year: 2025 (Filtered by Date Received)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add late fee waiver option and enhance payment dialog
- Introduced a checkbox in the Late Fee Dialog to waive late fees if rent is paid in full by the end of the month.
- Updated the configuration saving logic to include the new waiver option.
- Enhanced the Payment Dialog to display a summary of the selected month, including late fees and remaining balance.
- Improved the handling of payment notes to include automatic late-payment notes.
- Refactored the Rent Management Tab to incorporate the new late fee waiver logic and display relevant information in the payment history and monthly summaries.
- Added functionality to export late fee history in CSV format.
</commit_message>
<xml_diff>
--- a/Financial Manager/resources/Maria(Current)_rent_export.xlsx
+++ b/Financial Manager/resources/Maria(Current)_rent_export.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Main'!$A$1:$H$74</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'2026'!$A$1:$H$37</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Main'!$A$1:$H$77</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'2026'!$A$1:$H$40</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'2025'!$A$1:$H$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -64,7 +64,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -115,6 +115,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F8F4E8"/>
         <bgColor rgb="00F8F4E8"/>
       </patternFill>
@@ -145,8 +151,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-        <bgColor rgb="00FFEB9C"/>
+        <fgColor rgb="009CC2E5"/>
+        <bgColor rgb="009CC2E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+        <bgColor rgb="00FF0000"/>
       </patternFill>
     </fill>
     <fill>
@@ -186,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -221,22 +233,22 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -248,46 +260,52 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="19" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -655,7 +673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -664,14 +682,14 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Report Generated: 2026-04-02 23:23:07</t>
+          <t>Report Generated: 2026-05-22 20:42:57</t>
         </is>
       </c>
     </row>
@@ -792,7 +810,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>April 2026</t>
+          <t>May 2026</t>
         </is>
       </c>
     </row>
@@ -835,7 +853,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>1850</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="20">
@@ -865,7 +883,7 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>1850</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="24">
@@ -1024,18 +1042,22 @@
           <t>2025-03</t>
         </is>
       </c>
-      <c r="E29" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F29" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2025-03-02</t>
         </is>
       </c>
       <c r="G29" s="11" t="inlineStr"/>
-      <c r="H29" s="12" t="inlineStr"/>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-03-02</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n">
@@ -1049,7 +1071,7 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D30" s="17" t="inlineStr">
+      <c r="D30" s="18" t="inlineStr">
         <is>
           <t>2025-04</t>
         </is>
@@ -1079,23 +1101,27 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D31" s="18" t="inlineStr">
+      <c r="D31" s="19" t="inlineStr">
         <is>
           <t>2025-05</t>
         </is>
       </c>
-      <c r="E31" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F31" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2026-01-29</t>
         </is>
       </c>
       <c r="G31" s="11" t="inlineStr"/>
-      <c r="H31" s="12" t="inlineStr"/>
+      <c r="H31" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-01-29</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n">
@@ -1109,89 +1135,93 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D32" s="18" t="inlineStr">
+      <c r="D32" s="19" t="inlineStr">
         <is>
           <t>2025-05</t>
         </is>
       </c>
-      <c r="E32" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F32" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2026-01-29</t>
         </is>
       </c>
       <c r="G32" s="11" t="inlineStr"/>
-      <c r="H32" s="12" t="inlineStr"/>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-01-29</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="19" t="n">
+      <c r="A33" s="20" t="n">
         <v>46051</v>
       </c>
-      <c r="B33" s="20" t="n">
+      <c r="B33" s="21" t="n">
         <v>100</v>
       </c>
-      <c r="C33" s="21" t="inlineStr">
+      <c r="C33" s="22" t="inlineStr">
         <is>
           <t>Overpayment Credit (Applied: $100.00)</t>
         </is>
       </c>
-      <c r="D33" s="21" t="inlineStr">
+      <c r="D33" s="22" t="inlineStr">
         <is>
           <t>2025-05</t>
         </is>
       </c>
-      <c r="E33" s="21" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
-        </is>
-      </c>
-      <c r="F33" s="21" t="inlineStr">
-        <is>
-          <t>Fully paid</t>
-        </is>
-      </c>
-      <c r="G33" s="20" t="inlineStr"/>
-      <c r="H33" s="21" t="inlineStr">
-        <is>
-          <t>RANDOM MONTH TO PAY OFF</t>
+      <c r="E33" s="22" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
+        </is>
+      </c>
+      <c r="F33" s="22" t="inlineStr">
+        <is>
+          <t>Fully paid | Paid after due date on 2026-01-29</t>
+        </is>
+      </c>
+      <c r="G33" s="21" t="inlineStr"/>
+      <c r="H33" s="22" t="inlineStr">
+        <is>
+          <t>RANDOM MONTH TO PAY OFF | Paid after due date on 2026-01-29</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="19" t="n">
+      <c r="A34" s="20" t="n">
         <v>46051</v>
       </c>
-      <c r="B34" s="20" t="n">
+      <c r="B34" s="21" t="n">
         <v>50</v>
       </c>
-      <c r="C34" s="21" t="inlineStr">
+      <c r="C34" s="22" t="inlineStr">
         <is>
           <t>Overpayment Credit (Applied: $50.00)</t>
         </is>
       </c>
-      <c r="D34" s="21" t="inlineStr">
+      <c r="D34" s="22" t="inlineStr">
         <is>
           <t>2025-05</t>
         </is>
       </c>
-      <c r="E34" s="21" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
-        </is>
-      </c>
-      <c r="F34" s="21" t="inlineStr">
-        <is>
-          <t>Fully paid</t>
-        </is>
-      </c>
-      <c r="G34" s="20" t="inlineStr"/>
-      <c r="H34" s="21" t="inlineStr">
-        <is>
-          <t>RANDOM MONTH TO PAY OFF</t>
+      <c r="E34" s="22" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
+        </is>
+      </c>
+      <c r="F34" s="22" t="inlineStr">
+        <is>
+          <t>Fully paid | Paid after due date on 2026-01-29</t>
+        </is>
+      </c>
+      <c r="G34" s="21" t="inlineStr"/>
+      <c r="H34" s="22" t="inlineStr">
+        <is>
+          <t>RANDOM MONTH TO PAY OFF | Paid after due date on 2026-01-29</t>
         </is>
       </c>
     </row>
@@ -1212,12 +1242,12 @@
           <t>2025-06</t>
         </is>
       </c>
-      <c r="E35" s="22" t="inlineStr">
+      <c r="E35" s="23" t="inlineStr">
         <is>
           <t>Overpayment</t>
         </is>
       </c>
-      <c r="F35" s="22" t="inlineStr">
+      <c r="F35" s="23" t="inlineStr">
         <is>
           <t>Overpaid by $150.00</t>
         </is>
@@ -1242,12 +1272,12 @@
           <t>2025-06</t>
         </is>
       </c>
-      <c r="E36" s="22" t="inlineStr">
+      <c r="E36" s="23" t="inlineStr">
         <is>
           <t>Overpayment</t>
         </is>
       </c>
-      <c r="F36" s="22" t="inlineStr">
+      <c r="F36" s="23" t="inlineStr">
         <is>
           <t>Overpaid by $150.00</t>
         </is>
@@ -1274,18 +1304,22 @@
           <t>2025-07</t>
         </is>
       </c>
-      <c r="E37" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F37" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2025-07-31</t>
         </is>
       </c>
       <c r="G37" s="11" t="inlineStr"/>
-      <c r="H37" s="12" t="inlineStr"/>
+      <c r="H37" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-07-31</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n">
@@ -1304,18 +1338,22 @@
           <t>2025-07</t>
         </is>
       </c>
-      <c r="E38" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E38" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F38" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2025-07-31</t>
         </is>
       </c>
       <c r="G38" s="11" t="inlineStr"/>
-      <c r="H38" s="12" t="inlineStr"/>
+      <c r="H38" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-07-31</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="10" t="n">
@@ -1334,18 +1372,22 @@
           <t>2025-07</t>
         </is>
       </c>
-      <c r="E39" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E39" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F39" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2025-07-31</t>
         </is>
       </c>
       <c r="G39" s="11" t="inlineStr"/>
-      <c r="H39" s="12" t="inlineStr"/>
+      <c r="H39" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-07-31</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n">
@@ -1364,18 +1406,22 @@
           <t>2025-07</t>
         </is>
       </c>
-      <c r="E40" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E40" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F40" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2025-07-31</t>
         </is>
       </c>
       <c r="G40" s="11" t="inlineStr"/>
-      <c r="H40" s="12" t="inlineStr"/>
+      <c r="H40" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-07-31</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="n">
@@ -1394,18 +1440,22 @@
           <t>2025-08</t>
         </is>
       </c>
-      <c r="E41" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F41" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $50.00</t>
+      <c r="E41" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F41" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $50.00 | Paid after due date on 2025-08-24</t>
         </is>
       </c>
       <c r="G41" s="11" t="inlineStr"/>
-      <c r="H41" s="12" t="inlineStr"/>
+      <c r="H41" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-08-24</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n">
@@ -1424,20 +1474,24 @@
           <t>2025-08</t>
         </is>
       </c>
-      <c r="E42" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F42" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $50.00</t>
+      <c r="E42" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F42" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $50.00 | Paid after due date on 2025-08-24</t>
         </is>
       </c>
       <c r="G42" s="11" t="n">
         <v>50</v>
       </c>
-      <c r="H42" s="12" t="inlineStr"/>
+      <c r="H42" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-08-24</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="10" t="n">
@@ -1451,23 +1505,27 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D43" s="17" t="inlineStr">
+      <c r="D43" s="18" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
       </c>
-      <c r="E43" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F43" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $800.00</t>
+      <c r="E43" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F43" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $800.00 | Paid after due date on 2026-03-07</t>
         </is>
       </c>
       <c r="G43" s="11" t="inlineStr"/>
-      <c r="H43" s="12" t="inlineStr"/>
+      <c r="H43" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-03-07</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n">
@@ -1481,23 +1539,27 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D44" s="17" t="inlineStr">
+      <c r="D44" s="18" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
       </c>
-      <c r="E44" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F44" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $800.00</t>
+      <c r="E44" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F44" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $800.00 | Paid after due date on 2026-03-07</t>
         </is>
       </c>
       <c r="G44" s="11" t="inlineStr"/>
-      <c r="H44" s="12" t="inlineStr"/>
+      <c r="H44" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-03-07</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="n">
@@ -1511,157 +1573,161 @@
           <t>Cash</t>
         </is>
       </c>
-      <c r="D45" s="17" t="inlineStr">
+      <c r="D45" s="18" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
       </c>
-      <c r="E45" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F45" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $800.00</t>
+      <c r="E45" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F45" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $800.00 | Paid after due date on 2026-03-07</t>
         </is>
       </c>
       <c r="G45" s="11" t="inlineStr"/>
-      <c r="H45" s="12" t="inlineStr"/>
+      <c r="H45" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-03-07</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="19" t="n">
+      <c r="A46" s="20" t="n">
         <v>46030</v>
       </c>
-      <c r="B46" s="20" t="n">
+      <c r="B46" s="21" t="n">
         <v>100</v>
       </c>
-      <c r="C46" s="21" t="inlineStr">
+      <c r="C46" s="22" t="inlineStr">
         <is>
           <t>Overpayment Credit (Applied: $100.00)</t>
         </is>
       </c>
-      <c r="D46" s="21" t="inlineStr">
+      <c r="D46" s="22" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
       </c>
-      <c r="E46" s="21" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F46" s="21" t="inlineStr">
-        <is>
-          <t>Overpaid by $800.00</t>
-        </is>
-      </c>
-      <c r="G46" s="20" t="inlineStr"/>
-      <c r="H46" s="21" t="inlineStr">
-        <is>
-          <t>Random Month</t>
+      <c r="E46" s="22" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F46" s="22" t="inlineStr">
+        <is>
+          <t>Overpaid by $800.00 | Paid after due date on 2026-03-07</t>
+        </is>
+      </c>
+      <c r="G46" s="21" t="inlineStr"/>
+      <c r="H46" s="22" t="inlineStr">
+        <is>
+          <t>Random Month | Paid after due date on 2026-03-07</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="19" t="n">
+      <c r="A47" s="20" t="n">
         <v>46030</v>
       </c>
-      <c r="B47" s="20" t="n">
+      <c r="B47" s="21" t="n">
         <v>150</v>
       </c>
-      <c r="C47" s="21" t="inlineStr">
+      <c r="C47" s="22" t="inlineStr">
         <is>
           <t>Overpayment Credit (Applied: $150.00)</t>
         </is>
       </c>
-      <c r="D47" s="21" t="inlineStr">
+      <c r="D47" s="22" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
       </c>
-      <c r="E47" s="21" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F47" s="21" t="inlineStr">
-        <is>
-          <t>Overpaid by $800.00</t>
-        </is>
-      </c>
-      <c r="G47" s="20" t="inlineStr"/>
-      <c r="H47" s="21" t="inlineStr">
-        <is>
-          <t>Random Month Chosen</t>
+      <c r="E47" s="22" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F47" s="22" t="inlineStr">
+        <is>
+          <t>Overpaid by $800.00 | Paid after due date on 2026-03-07</t>
+        </is>
+      </c>
+      <c r="G47" s="21" t="inlineStr"/>
+      <c r="H47" s="22" t="inlineStr">
+        <is>
+          <t>Random Month Chosen | Paid after due date on 2026-03-07</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="19" t="n">
+      <c r="A48" s="20" t="n">
         <v>46051</v>
       </c>
-      <c r="B48" s="20" t="n">
+      <c r="B48" s="21" t="n">
         <v>50</v>
       </c>
-      <c r="C48" s="21" t="inlineStr">
+      <c r="C48" s="22" t="inlineStr">
         <is>
           <t>Overpayment Credit (Applied: $50.00)</t>
         </is>
       </c>
-      <c r="D48" s="21" t="inlineStr">
+      <c r="D48" s="22" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
       </c>
-      <c r="E48" s="21" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F48" s="21" t="inlineStr">
-        <is>
-          <t>Overpaid by $800.00</t>
-        </is>
-      </c>
-      <c r="G48" s="20" t="inlineStr"/>
-      <c r="H48" s="21" t="inlineStr">
-        <is>
-          <t>RANDOM MONTH TO APPLY</t>
+      <c r="E48" s="22" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F48" s="22" t="inlineStr">
+        <is>
+          <t>Overpaid by $800.00 | Paid after due date on 2026-03-07</t>
+        </is>
+      </c>
+      <c r="G48" s="21" t="inlineStr"/>
+      <c r="H48" s="22" t="inlineStr">
+        <is>
+          <t>RANDOM MONTH TO APPLY | Paid after due date on 2026-03-07</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="19" t="n">
+      <c r="A49" s="20" t="n">
         <v>46057</v>
       </c>
-      <c r="B49" s="20" t="n">
+      <c r="B49" s="21" t="n">
         <v>150</v>
       </c>
-      <c r="C49" s="21" t="inlineStr">
+      <c r="C49" s="22" t="inlineStr">
         <is>
           <t>Overpayment Credit (Applied: $150.00)</t>
         </is>
       </c>
-      <c r="D49" s="21" t="inlineStr">
+      <c r="D49" s="22" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
       </c>
-      <c r="E49" s="21" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F49" s="21" t="inlineStr">
-        <is>
-          <t>Overpaid by $800.00</t>
-        </is>
-      </c>
-      <c r="G49" s="20" t="inlineStr"/>
-      <c r="H49" s="21" t="inlineStr">
-        <is>
-          <t>RANDOM ASSIGNED</t>
+      <c r="E49" s="22" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F49" s="22" t="inlineStr">
+        <is>
+          <t>Overpaid by $800.00 | Paid after due date on 2026-03-07</t>
+        </is>
+      </c>
+      <c r="G49" s="21" t="inlineStr"/>
+      <c r="H49" s="22" t="inlineStr">
+        <is>
+          <t>RANDOM ASSIGNED | Paid after due date on 2026-03-07</t>
         </is>
       </c>
     </row>
@@ -1677,19 +1743,19 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D50" s="17" t="inlineStr">
+      <c r="D50" s="18" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
       </c>
-      <c r="E50" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F50" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $800.00</t>
+      <c r="E50" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F50" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $800.00 | Paid after due date on 2026-03-07</t>
         </is>
       </c>
       <c r="G50" s="11" t="n">
@@ -1697,7 +1763,7 @@
       </c>
       <c r="H50" s="12" t="inlineStr">
         <is>
-          <t>2 payments of 500 $ targeted to pay off random delinquent months</t>
+          <t>2 payments of 500 $ targeted to pay off random delinquent months | Paid after due date on 2026-03-07</t>
         </is>
       </c>
     </row>
@@ -1718,18 +1784,22 @@
           <t>2025-10</t>
         </is>
       </c>
-      <c r="E51" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F51" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $200.00</t>
+      <c r="E51" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F51" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00 | Paid after due date on 2026-01-13</t>
         </is>
       </c>
       <c r="G51" s="11" t="inlineStr"/>
-      <c r="H51" s="12" t="inlineStr"/>
+      <c r="H51" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="10" t="n">
@@ -1748,18 +1818,22 @@
           <t>2025-10</t>
         </is>
       </c>
-      <c r="E52" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F52" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $200.00</t>
+      <c r="E52" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F52" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00 | Paid after due date on 2026-01-13</t>
         </is>
       </c>
       <c r="G52" s="11" t="inlineStr"/>
-      <c r="H52" s="12" t="inlineStr"/>
+      <c r="H52" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="10" t="n">
@@ -1778,14 +1852,14 @@
           <t>2025-10</t>
         </is>
       </c>
-      <c r="E53" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F53" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $200.00</t>
+      <c r="E53" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F53" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00 | Paid after due date on 2026-01-13</t>
         </is>
       </c>
       <c r="G53" s="11" t="n">
@@ -1793,7 +1867,7 @@
       </c>
       <c r="H53" s="12" t="inlineStr">
         <is>
-          <t>RANDOM MONTH TO PAY OFF</t>
+          <t>RANDOM MONTH TO PAY OFF | Paid after due date on 2026-01-13</t>
         </is>
       </c>
     </row>
@@ -1814,18 +1888,22 @@
           <t>2025-11</t>
         </is>
       </c>
-      <c r="E54" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F54" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $50.00</t>
+      <c r="E54" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F54" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $50.00 | Paid after due date on 2026-01-07</t>
         </is>
       </c>
       <c r="G54" s="11" t="inlineStr"/>
-      <c r="H54" s="12" t="inlineStr"/>
+      <c r="H54" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-01-07</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="10" t="n">
@@ -1844,20 +1922,24 @@
           <t>2025-11</t>
         </is>
       </c>
-      <c r="E55" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F55" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $50.00</t>
+      <c r="E55" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F55" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $50.00 | Paid after due date on 2026-01-07</t>
         </is>
       </c>
       <c r="G55" s="11" t="n">
         <v>50</v>
       </c>
-      <c r="H55" s="12" t="inlineStr"/>
+      <c r="H55" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-01-07</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="10" t="n">
@@ -1871,55 +1953,59 @@
           <t>Cash</t>
         </is>
       </c>
-      <c r="D56" s="18" t="inlineStr">
+      <c r="D56" s="19" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
       </c>
-      <c r="E56" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E56" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F56" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2026-03-07</t>
         </is>
       </c>
       <c r="G56" s="11" t="inlineStr"/>
-      <c r="H56" s="12" t="inlineStr"/>
+      <c r="H56" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-03-07</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="19" t="n">
+      <c r="A57" s="20" t="n">
         <v>46088</v>
       </c>
-      <c r="B57" s="20" t="n">
+      <c r="B57" s="21" t="n">
         <v>350</v>
       </c>
-      <c r="C57" s="21" t="inlineStr">
+      <c r="C57" s="22" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="D57" s="21" t="inlineStr">
+      <c r="D57" s="22" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
       </c>
-      <c r="E57" s="21" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
-        </is>
-      </c>
-      <c r="F57" s="21" t="inlineStr">
-        <is>
-          <t>Fully paid</t>
-        </is>
-      </c>
-      <c r="G57" s="20" t="inlineStr"/>
-      <c r="H57" s="21" t="inlineStr">
-        <is>
-          <t>RANDOM TARGETED MONTH TO PAY OFF</t>
+      <c r="E57" s="22" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
+        </is>
+      </c>
+      <c r="F57" s="22" t="inlineStr">
+        <is>
+          <t>Fully paid | Paid after due date on 2026-03-07</t>
+        </is>
+      </c>
+      <c r="G57" s="21" t="inlineStr"/>
+      <c r="H57" s="22" t="inlineStr">
+        <is>
+          <t>RANDOM TARGETED MONTH TO PAY OFF | Paid after due date on 2026-03-07</t>
         </is>
       </c>
     </row>
@@ -1940,52 +2026,56 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="E58" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F58" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $150.00</t>
+      <c r="E58" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F58" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $150.00 | Paid after due date on 2026-02-04</t>
         </is>
       </c>
       <c r="G58" s="11" t="n">
         <v>150</v>
       </c>
-      <c r="H58" s="12" t="inlineStr"/>
+      <c r="H58" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-02-04</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="19" t="n">
+      <c r="A59" s="20" t="n">
         <v>46088</v>
       </c>
-      <c r="B59" s="20" t="n">
+      <c r="B59" s="21" t="n">
         <v>450</v>
       </c>
-      <c r="C59" s="21" t="inlineStr">
+      <c r="C59" s="22" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="D59" s="21" t="inlineStr">
+      <c r="D59" s="22" t="inlineStr">
         <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="E59" s="21" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F59" s="21" t="inlineStr">
-        <is>
-          <t>Overpaid by $200.00</t>
-        </is>
-      </c>
-      <c r="G59" s="20" t="inlineStr"/>
-      <c r="H59" s="21" t="inlineStr">
-        <is>
-          <t>RANDOM TARGETED MONTH TO APPLY OVERCREDIT</t>
+      <c r="E59" s="22" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F59" s="22" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00 | Paid after due date on 2026-04-01</t>
+        </is>
+      </c>
+      <c r="G59" s="21" t="inlineStr"/>
+      <c r="H59" s="22" t="inlineStr">
+        <is>
+          <t>RANDOM TARGETED MONTH TO APPLY OVERCREDIT | Paid after due date on 2026-04-01</t>
         </is>
       </c>
     </row>
@@ -2001,23 +2091,27 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D60" s="17" t="inlineStr">
+      <c r="D60" s="18" t="inlineStr">
         <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="E60" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F60" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $200.00</t>
+      <c r="E60" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F60" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00 | Paid after due date on 2026-04-01</t>
         </is>
       </c>
       <c r="G60" s="11" t="inlineStr"/>
-      <c r="H60" s="12" t="inlineStr"/>
+      <c r="H60" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-04-01</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="10" t="n">
@@ -2031,25 +2125,29 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D61" s="17" t="inlineStr">
+      <c r="D61" s="18" t="inlineStr">
         <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="E61" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F61" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $200.00</t>
+      <c r="E61" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F61" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00 | Paid after due date on 2026-04-01</t>
         </is>
       </c>
       <c r="G61" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="H61" s="12" t="inlineStr"/>
+      <c r="H61" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-04-01</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="10" t="n">
@@ -2063,266 +2161,422 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D62" s="18" t="inlineStr">
+      <c r="D62" s="19" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="E62" s="23" t="inlineStr">
-        <is>
-          <t>Partial Payment</t>
-        </is>
-      </c>
-      <c r="F62" s="24" t="inlineStr">
-        <is>
-          <t>$500.00 remaining</t>
+      <c r="E62" s="25" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
+        </is>
+      </c>
+      <c r="F62" s="26" t="inlineStr">
+        <is>
+          <t>$250.00 remaining | Late and still owes $250.00</t>
         </is>
       </c>
       <c r="G62" s="11" t="inlineStr"/>
-      <c r="H62" s="12" t="inlineStr"/>
+      <c r="H62" s="12" t="inlineStr">
+        <is>
+          <t>Late and still owes $250.00</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="19" t="n">
+      <c r="A63" s="20" t="n">
         <v>46114</v>
       </c>
-      <c r="B63" s="20" t="n">
+      <c r="B63" s="21" t="n">
         <v>200</v>
       </c>
-      <c r="C63" s="21" t="inlineStr">
+      <c r="C63" s="22" t="inlineStr">
         <is>
           <t>Overpayment Credit (Applied: $200.00)</t>
         </is>
       </c>
-      <c r="D63" s="21" t="inlineStr">
+      <c r="D63" s="22" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="E63" s="21" t="inlineStr">
-        <is>
-          <t>Partial Payment</t>
-        </is>
-      </c>
-      <c r="F63" s="21" t="inlineStr">
-        <is>
-          <t>$500.00 remaining</t>
-        </is>
-      </c>
-      <c r="G63" s="20" t="inlineStr"/>
-      <c r="H63" s="21" t="inlineStr">
-        <is>
-          <t>Random applied to current month</t>
+      <c r="E63" s="22" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
+        </is>
+      </c>
+      <c r="F63" s="22" t="inlineStr">
+        <is>
+          <t>$250.00 remaining | Late and still owes $250.00</t>
+        </is>
+      </c>
+      <c r="G63" s="21" t="inlineStr"/>
+      <c r="H63" s="22" t="inlineStr">
+        <is>
+          <t>Random applied to current month | Late and still owes $250.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="n">
+        <v>46116</v>
+      </c>
+      <c r="B64" s="11" t="n">
+        <v>250</v>
+      </c>
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>Zelle</t>
+        </is>
+      </c>
+      <c r="D64" s="19" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="E64" s="25" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
+        </is>
+      </c>
+      <c r="F64" s="26" t="inlineStr">
+        <is>
+          <t>$250.00 remaining | Late and still owes $250.00</t>
+        </is>
+      </c>
+      <c r="G64" s="11" t="inlineStr"/>
+      <c r="H64" s="12" t="inlineStr">
+        <is>
+          <t>Applied for Delinquet month | Late and still owes $250.00</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="inlineStr">
+      <c r="A65" s="10" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B65" s="11" t="n">
+        <v>1300</v>
+      </c>
+      <c r="C65" s="12" t="inlineStr">
+        <is>
+          <t>Zelle</t>
+        </is>
+      </c>
+      <c r="D65" s="13" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="E65" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
+        </is>
+      </c>
+      <c r="F65" s="14" t="inlineStr">
+        <is>
+          <t>Fully paid | Paid after due date on 2026-05-22</t>
+        </is>
+      </c>
+      <c r="G65" s="11" t="inlineStr"/>
+      <c r="H65" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-05-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B66" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="C66" s="12" t="inlineStr">
+        <is>
+          <t>Zelle</t>
+        </is>
+      </c>
+      <c r="D66" s="13" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="E66" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
+        </is>
+      </c>
+      <c r="F66" s="14" t="inlineStr">
+        <is>
+          <t>Fully paid | Paid after due date on 2026-05-22</t>
+        </is>
+      </c>
+      <c r="G66" s="11" t="inlineStr"/>
+      <c r="H66" s="12" t="inlineStr">
+        <is>
+          <t>Late | Paid after due date on 2026-05-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
         <is>
           <t>MONTHLY BALANCE SUMMARY (Filtered)</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="9" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="9" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B66" s="9" t="inlineStr">
+      <c r="B69" s="9" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C66" s="9" t="inlineStr">
+      <c r="C69" s="9" t="inlineStr">
         <is>
           <t>Rent Due</t>
         </is>
       </c>
-      <c r="D66" s="9" t="inlineStr">
+      <c r="D69" s="9" t="inlineStr">
         <is>
           <t>Total Paid</t>
         </is>
       </c>
-      <c r="E66" s="9" t="inlineStr">
+      <c r="E69" s="9" t="inlineStr">
         <is>
           <t>Balance</t>
         </is>
       </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="25" t="inlineStr">
+      <c r="F69" s="9" t="inlineStr">
+        <is>
+          <t>Late Fees</t>
+        </is>
+      </c>
+      <c r="G69" s="9" t="inlineStr">
+        <is>
+          <t>Late Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="27" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="B67" s="26" t="inlineStr">
-        <is>
-          <t>Partial Payment</t>
-        </is>
-      </c>
-      <c r="C67" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D67" s="27" t="n">
-        <v>850</v>
-      </c>
-      <c r="E67" s="28" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="25" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B68" s="29" t="inlineStr">
-        <is>
-          <t>Not Paid</t>
-        </is>
-      </c>
-      <c r="C68" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D68" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E68" s="30" t="n">
-        <v>1350</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="25" t="inlineStr">
+      <c r="B70" s="28" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
+        </is>
+      </c>
+      <c r="C70" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D70" s="29" t="n">
+        <v>1100</v>
+      </c>
+      <c r="E70" s="30" t="n">
+        <v>250</v>
+      </c>
+      <c r="F70" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="27" t="inlineStr">
+        <is>
+          <t>Late and still owes $250.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="27" t="inlineStr">
         <is>
           <t>2026-05</t>
         </is>
       </c>
-      <c r="B69" s="31" t="inlineStr">
+      <c r="B71" s="28" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
+        </is>
+      </c>
+      <c r="C71" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D71" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" s="30" t="n">
+        <v>1350</v>
+      </c>
+      <c r="F71" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" s="27" t="inlineStr">
+        <is>
+          <t>Late and still owes $1350.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="27" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B72" s="31" t="inlineStr">
         <is>
           <t>Due Soon</t>
         </is>
       </c>
-      <c r="C69" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D69" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E69" s="32" t="n">
-        <v>1350</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="25" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B70" s="33" t="inlineStr">
+      <c r="C72" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D72" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="32" t="n">
+        <v>1350</v>
+      </c>
+      <c r="F72" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="27" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="27" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B73" s="33" t="inlineStr">
         <is>
           <t>Not Due</t>
         </is>
       </c>
-      <c r="C70" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D70" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E70" s="34" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="25" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B71" s="33" t="inlineStr">
+      <c r="C73" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D73" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="27" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="27" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B74" s="33" t="inlineStr">
         <is>
           <t>Not Due</t>
         </is>
       </c>
-      <c r="C71" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D71" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E71" s="34" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="25" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B72" s="33" t="inlineStr">
+      <c r="C74" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D74" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="27" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="27" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B75" s="33" t="inlineStr">
         <is>
           <t>Not Due</t>
         </is>
       </c>
-      <c r="C72" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D72" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E72" s="34" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="25" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B73" s="33" t="inlineStr">
+      <c r="C75" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D75" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="27" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="27" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B76" s="33" t="inlineStr">
         <is>
           <t>Not Due</t>
         </is>
       </c>
-      <c r="C73" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D73" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E73" s="34" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="25" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="B74" s="33" t="inlineStr">
+      <c r="C76" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D76" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="27" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="27" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B77" s="33" t="inlineStr">
         <is>
           <t>Not Due</t>
         </is>
       </c>
-      <c r="C74" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D74" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E74" s="34" t="n">
-        <v>0</v>
-      </c>
+      <c r="C77" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D77" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="27" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A65:H65"/>
     <mergeCell ref="A24:H24"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A68:H68"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -2338,7 +2592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2347,14 +2601,14 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Report Generated: 2026-04-02 23:23:09 | Year: 2026 (Filtered by Payment Month)</t>
+          <t>Report Generated: 2026-05-22 20:42:58 | Year: 2026 (Filtered by Payment Month)</t>
         </is>
       </c>
     </row>
@@ -2484,52 +2738,56 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="E12" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F12" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $150.00</t>
+      <c r="E12" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F12" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $150.00 | Paid after due date on 2026-02-04</t>
         </is>
       </c>
       <c r="G12" s="11" t="n">
         <v>150</v>
       </c>
-      <c r="H12" s="12" t="inlineStr"/>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-02-04</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n">
+      <c r="A13" s="20" t="n">
         <v>46088</v>
       </c>
-      <c r="B13" s="20" t="n">
+      <c r="B13" s="21" t="n">
         <v>450</v>
       </c>
-      <c r="C13" s="21" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="D13" s="21" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="E13" s="21" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F13" s="21" t="inlineStr">
-        <is>
-          <t>Overpaid by $200.00</t>
-        </is>
-      </c>
-      <c r="G13" s="20" t="inlineStr"/>
-      <c r="H13" s="21" t="inlineStr">
-        <is>
-          <t>RANDOM TARGETED MONTH TO APPLY OVERCREDIT</t>
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F13" s="22" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00 | Paid after due date on 2026-04-01</t>
+        </is>
+      </c>
+      <c r="G13" s="21" t="inlineStr"/>
+      <c r="H13" s="22" t="inlineStr">
+        <is>
+          <t>RANDOM TARGETED MONTH TO APPLY OVERCREDIT | Paid after due date on 2026-04-01</t>
         </is>
       </c>
     </row>
@@ -2545,23 +2803,27 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D14" s="17" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="E14" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F14" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $200.00</t>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00 | Paid after due date on 2026-04-01</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr"/>
-      <c r="H14" s="12" t="inlineStr"/>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-04-01</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="n">
@@ -2575,25 +2837,29 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D15" s="17" t="inlineStr">
+      <c r="D15" s="18" t="inlineStr">
         <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="E15" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F15" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $200.00</t>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00 | Paid after due date on 2026-04-01</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="H15" s="12" t="inlineStr"/>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-04-01</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n">
@@ -2607,389 +2873,573 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="D16" s="19" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="E16" s="23" t="inlineStr">
-        <is>
-          <t>Partial Payment</t>
-        </is>
-      </c>
-      <c r="F16" s="24" t="inlineStr">
-        <is>
-          <t>$500.00 remaining</t>
+      <c r="E16" s="25" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>$250.00 remaining | Late and still owes $250.00</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr"/>
-      <c r="H16" s="12" t="inlineStr"/>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>Late and still owes $250.00</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="n">
+      <c r="A17" s="20" t="n">
         <v>46114</v>
       </c>
-      <c r="B17" s="20" t="n">
+      <c r="B17" s="21" t="n">
         <v>200</v>
       </c>
-      <c r="C17" s="21" t="inlineStr">
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>Overpayment Credit (Applied: $200.00)</t>
         </is>
       </c>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="D17" s="22" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="E17" s="21" t="inlineStr">
-        <is>
-          <t>Partial Payment</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="inlineStr">
-        <is>
-          <t>$500.00 remaining</t>
-        </is>
-      </c>
-      <c r="G17" s="20" t="inlineStr"/>
-      <c r="H17" s="21" t="inlineStr">
-        <is>
-          <t>Random applied to current month</t>
+      <c r="E17" s="22" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
+        </is>
+      </c>
+      <c r="F17" s="22" t="inlineStr">
+        <is>
+          <t>$250.00 remaining | Late and still owes $250.00</t>
+        </is>
+      </c>
+      <c r="G17" s="21" t="inlineStr"/>
+      <c r="H17" s="22" t="inlineStr">
+        <is>
+          <t>Random applied to current month | Late and still owes $250.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="n">
+        <v>46116</v>
+      </c>
+      <c r="B18" s="11" t="n">
+        <v>250</v>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Zelle</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="E18" s="25" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>$250.00 remaining | Late and still owes $250.00</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr"/>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>Applied for Delinquet month | Late and still owes $250.00</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="10" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>1300</v>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Zelle</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>Fully paid | Paid after due date on 2026-05-22</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr"/>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-05-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Zelle</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
+        </is>
+      </c>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>Fully paid | Paid after due date on 2026-05-22</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr"/>
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>Late | Paid after due date on 2026-05-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>YEAR SUMMARY - 2026 (Tax Purposes)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Total Actual Payments</t>
         </is>
       </c>
-      <c r="B20" s="35" t="n">
-        <v>3250</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="B23" s="35" t="n">
+        <v>4850</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Total Rent Due</t>
         </is>
       </c>
-      <c r="B21" s="36" t="n">
+      <c r="B24" s="36" t="n">
         <v>16200</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Net Difference</t>
         </is>
       </c>
-      <c r="B22" s="37" t="n">
-        <v>-12950</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="B25" s="37" t="n">
+        <v>-11350</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>MONTHLY BALANCE SUMMARY - 2026</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>Rent Due</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>Total Paid</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr">
         <is>
           <t>Balance</t>
         </is>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="25" t="inlineStr">
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Late Fees</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>Late Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="27" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
       </c>
-      <c r="B26" s="38" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="C26" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D26" s="27" t="n">
+      <c r="B29" s="38" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="C29" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D29" s="29" t="n">
         <v>1500</v>
       </c>
-      <c r="E26" s="39" t="n">
+      <c r="E29" s="39" t="n">
         <v>-150</v>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="25" t="inlineStr">
+      <c r="F29" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="27" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-02-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="27" t="inlineStr">
         <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="B27" s="38" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="C27" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D27" s="27" t="n">
+      <c r="B30" s="38" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="C30" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D30" s="29" t="n">
         <v>1550</v>
       </c>
-      <c r="E27" s="39" t="n">
+      <c r="E30" s="39" t="n">
         <v>-200</v>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="25" t="inlineStr">
+      <c r="F30" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="27" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-04-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="27" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="B28" s="26" t="inlineStr">
-        <is>
-          <t>Partial Payment</t>
-        </is>
-      </c>
-      <c r="C28" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D28" s="27" t="n">
-        <v>850</v>
-      </c>
-      <c r="E28" s="28" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="25" t="inlineStr">
+      <c r="B31" s="28" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
+        </is>
+      </c>
+      <c r="C31" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D31" s="29" t="n">
+        <v>1100</v>
+      </c>
+      <c r="E31" s="30" t="n">
+        <v>250</v>
+      </c>
+      <c r="F31" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="27" t="inlineStr">
+        <is>
+          <t>Late and still owes $250.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="27" t="inlineStr">
         <is>
           <t>2026-04</t>
         </is>
       </c>
-      <c r="B29" s="29" t="inlineStr">
-        <is>
-          <t>Not Paid</t>
-        </is>
-      </c>
-      <c r="C29" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D29" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="30" t="n">
-        <v>1350</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="25" t="inlineStr">
+      <c r="B32" s="40" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
+        </is>
+      </c>
+      <c r="C32" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D32" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E32" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="27" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-05-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="27" t="inlineStr">
         <is>
           <t>2026-05</t>
         </is>
       </c>
-      <c r="B30" s="31" t="inlineStr">
+      <c r="B33" s="28" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
+        </is>
+      </c>
+      <c r="C33" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D33" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="30" t="n">
+        <v>1350</v>
+      </c>
+      <c r="F33" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="27" t="inlineStr">
+        <is>
+          <t>Late and still owes $1350.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="27" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B34" s="31" t="inlineStr">
         <is>
           <t>Due Soon</t>
         </is>
       </c>
-      <c r="C30" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D30" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="32" t="n">
-        <v>1350</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="25" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B31" s="33" t="inlineStr">
+      <c r="C34" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D34" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="32" t="n">
+        <v>1350</v>
+      </c>
+      <c r="F34" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="27" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="27" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B35" s="33" t="inlineStr">
         <is>
           <t>Not Due</t>
         </is>
       </c>
-      <c r="C31" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D31" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="34" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="25" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B32" s="33" t="inlineStr">
+      <c r="C35" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D35" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="27" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="27" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B36" s="33" t="inlineStr">
         <is>
           <t>Not Due</t>
         </is>
       </c>
-      <c r="C32" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D32" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" s="34" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="25" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B33" s="33" t="inlineStr">
+      <c r="C36" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D36" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="27" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="27" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B37" s="33" t="inlineStr">
         <is>
           <t>Not Due</t>
         </is>
       </c>
-      <c r="C33" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D33" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="34" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="25" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B34" s="33" t="inlineStr">
+      <c r="C37" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D37" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="27" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="27" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B38" s="33" t="inlineStr">
         <is>
           <t>Not Due</t>
         </is>
       </c>
-      <c r="C34" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D34" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="34" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="25" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="B35" s="33" t="inlineStr">
+      <c r="C38" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D38" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="27" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="27" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B39" s="33" t="inlineStr">
         <is>
           <t>Not Due</t>
         </is>
       </c>
-      <c r="C35" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D35" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" s="34" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="25" t="inlineStr">
-        <is>
-          <t>2026-11</t>
-        </is>
-      </c>
-      <c r="B36" s="33" t="inlineStr">
+      <c r="C39" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D39" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="27" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="27" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B40" s="33" t="inlineStr">
         <is>
           <t>Not Due</t>
         </is>
       </c>
-      <c r="C36" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D36" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" s="34" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="25" t="inlineStr">
-        <is>
-          <t>2026-12</t>
-        </is>
-      </c>
-      <c r="B37" s="33" t="inlineStr">
-        <is>
-          <t>Not Due</t>
-        </is>
-      </c>
-      <c r="C37" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D37" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" s="34" t="n">
-        <v>0</v>
-      </c>
+      <c r="C40" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D40" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="27" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A24:H24"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3012,14 +3462,14 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Report Generated: 2026-04-02 23:23:10 | Year: 2025 (Filtered by Date Received)</t>
+          <t>Report Generated: 2026-05-22 20:42:58 | Year: 2025 (Filtered by Date Received)</t>
         </is>
       </c>
     </row>
@@ -3239,18 +3689,22 @@
           <t>2025-03</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2025-03-02</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr"/>
-      <c r="H15" s="12" t="inlineStr"/>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-03-02</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n">
@@ -3264,7 +3718,7 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D16" s="17" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>2025-04</t>
         </is>
@@ -3294,23 +3748,27 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D17" s="18" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>2025-05</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2026-01-29</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr"/>
-      <c r="H17" s="12" t="inlineStr"/>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-01-29</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n">
@@ -3324,23 +3782,27 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>2025-05</t>
         </is>
       </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2026-01-29</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr"/>
-      <c r="H18" s="12" t="inlineStr"/>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-01-29</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="n">
@@ -3359,12 +3821,12 @@
           <t>2025-06</t>
         </is>
       </c>
-      <c r="E19" s="22" t="inlineStr">
+      <c r="E19" s="23" t="inlineStr">
         <is>
           <t>Overpayment</t>
         </is>
       </c>
-      <c r="F19" s="22" t="inlineStr">
+      <c r="F19" s="23" t="inlineStr">
         <is>
           <t>Overpaid by $150.00</t>
         </is>
@@ -3389,12 +3851,12 @@
           <t>2025-06</t>
         </is>
       </c>
-      <c r="E20" s="22" t="inlineStr">
+      <c r="E20" s="23" t="inlineStr">
         <is>
           <t>Overpayment</t>
         </is>
       </c>
-      <c r="F20" s="22" t="inlineStr">
+      <c r="F20" s="23" t="inlineStr">
         <is>
           <t>Overpaid by $150.00</t>
         </is>
@@ -3421,18 +3883,22 @@
           <t>2025-07</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2025-07-31</t>
         </is>
       </c>
       <c r="G21" s="11" t="inlineStr"/>
-      <c r="H21" s="12" t="inlineStr"/>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-07-31</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n">
@@ -3451,18 +3917,22 @@
           <t>2025-07</t>
         </is>
       </c>
-      <c r="E22" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2025-07-31</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr"/>
-      <c r="H22" s="12" t="inlineStr"/>
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-07-31</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n">
@@ -3481,18 +3951,22 @@
           <t>2025-07</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2025-07-31</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr"/>
-      <c r="H23" s="12" t="inlineStr"/>
+      <c r="H23" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-07-31</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n">
@@ -3511,18 +3985,22 @@
           <t>2025-07</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2025-07-31</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr"/>
-      <c r="H24" s="12" t="inlineStr"/>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-07-31</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="n">
@@ -3541,18 +4019,22 @@
           <t>2025-08</t>
         </is>
       </c>
-      <c r="E25" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F25" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $50.00</t>
+      <c r="E25" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F25" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $50.00 | Paid after due date on 2025-08-24</t>
         </is>
       </c>
       <c r="G25" s="11" t="inlineStr"/>
-      <c r="H25" s="12" t="inlineStr"/>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-08-24</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n">
@@ -3571,20 +4053,24 @@
           <t>2025-08</t>
         </is>
       </c>
-      <c r="E26" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F26" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $50.00</t>
+      <c r="E26" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F26" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $50.00 | Paid after due date on 2025-08-24</t>
         </is>
       </c>
       <c r="G26" s="11" t="n">
         <v>50</v>
       </c>
-      <c r="H26" s="12" t="inlineStr"/>
+      <c r="H26" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-08-24</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="n">
@@ -3598,23 +4084,27 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D27" s="17" t="inlineStr">
+      <c r="D27" s="18" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
       </c>
-      <c r="E27" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F27" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $800.00</t>
+      <c r="E27" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F27" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $800.00 | Paid after due date on 2026-03-07</t>
         </is>
       </c>
       <c r="G27" s="11" t="inlineStr"/>
-      <c r="H27" s="12" t="inlineStr"/>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-03-07</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n">
@@ -3628,23 +4118,27 @@
           <t>Zelle</t>
         </is>
       </c>
-      <c r="D28" s="17" t="inlineStr">
+      <c r="D28" s="18" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
       </c>
-      <c r="E28" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F28" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $800.00</t>
+      <c r="E28" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F28" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $800.00 | Paid after due date on 2026-03-07</t>
         </is>
       </c>
       <c r="G28" s="11" t="inlineStr"/>
-      <c r="H28" s="12" t="inlineStr"/>
+      <c r="H28" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-03-07</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="n">
@@ -3658,23 +4152,27 @@
           <t>Cash</t>
         </is>
       </c>
-      <c r="D29" s="17" t="inlineStr">
+      <c r="D29" s="18" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
       </c>
-      <c r="E29" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F29" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $800.00</t>
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F29" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $800.00 | Paid after due date on 2026-03-07</t>
         </is>
       </c>
       <c r="G29" s="11" t="inlineStr"/>
-      <c r="H29" s="12" t="inlineStr"/>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-03-07</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n">
@@ -3693,18 +4191,22 @@
           <t>2025-10</t>
         </is>
       </c>
-      <c r="E30" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F30" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $200.00</t>
+      <c r="E30" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F30" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00 | Paid after due date on 2026-01-13</t>
         </is>
       </c>
       <c r="G30" s="11" t="inlineStr"/>
-      <c r="H30" s="12" t="inlineStr"/>
+      <c r="H30" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="n">
@@ -3723,18 +4225,22 @@
           <t>2025-10</t>
         </is>
       </c>
-      <c r="E31" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F31" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $200.00</t>
+      <c r="E31" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F31" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $200.00 | Paid after due date on 2026-01-13</t>
         </is>
       </c>
       <c r="G31" s="11" t="inlineStr"/>
-      <c r="H31" s="12" t="inlineStr"/>
+      <c r="H31" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n">
@@ -3753,18 +4259,22 @@
           <t>2025-11</t>
         </is>
       </c>
-      <c r="E32" s="22" t="inlineStr">
-        <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="F32" s="22" t="inlineStr">
-        <is>
-          <t>Overpaid by $50.00</t>
+      <c r="E32" s="24" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="F32" s="23" t="inlineStr">
+        <is>
+          <t>Overpaid by $50.00 | Paid after due date on 2026-01-07</t>
         </is>
       </c>
       <c r="G32" s="11" t="inlineStr"/>
-      <c r="H32" s="12" t="inlineStr"/>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-01-07</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="n">
@@ -3778,23 +4288,27 @@
           <t>Cash</t>
         </is>
       </c>
-      <c r="D33" s="18" t="inlineStr">
+      <c r="D33" s="19" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
       </c>
-      <c r="E33" s="14" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="F33" s="14" t="inlineStr">
         <is>
-          <t>Fully paid</t>
+          <t>Fully paid | Paid after due date on 2026-03-07</t>
         </is>
       </c>
       <c r="G33" s="11" t="inlineStr"/>
-      <c r="H33" s="12" t="inlineStr"/>
+      <c r="H33" s="12" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-03-07</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -3866,257 +4380,347 @@
           <t>Balance</t>
         </is>
       </c>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>Late Fees</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>Late Note</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="25" t="inlineStr">
+      <c r="A42" s="27" t="inlineStr">
         <is>
           <t>2025-01</t>
         </is>
       </c>
-      <c r="B42" s="40" t="inlineStr">
+      <c r="B42" s="41" t="inlineStr">
         <is>
           <t>Paid in Full</t>
         </is>
       </c>
-      <c r="C42" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D42" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="E42" s="27" t="n">
-        <v>0</v>
-      </c>
+      <c r="C42" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D42" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E42" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="27" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="25" t="inlineStr">
+      <c r="A43" s="27" t="inlineStr">
         <is>
           <t>2025-02</t>
         </is>
       </c>
-      <c r="B43" s="40" t="inlineStr">
+      <c r="B43" s="41" t="inlineStr">
         <is>
           <t>Paid in Full</t>
         </is>
       </c>
-      <c r="C43" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D43" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="E43" s="27" t="n">
-        <v>0</v>
-      </c>
+      <c r="C43" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D43" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E43" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="27" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="25" t="inlineStr">
+      <c r="A44" s="27" t="inlineStr">
         <is>
           <t>2025-03</t>
         </is>
       </c>
       <c r="B44" s="40" t="inlineStr">
         <is>
+          <t>Paid Late</t>
+        </is>
+      </c>
+      <c r="C44" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D44" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E44" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="27" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-03-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="27" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B45" s="41" t="inlineStr">
+        <is>
           <t>Paid in Full</t>
         </is>
       </c>
-      <c r="C44" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D44" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="E44" s="27" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="25" t="inlineStr">
-        <is>
-          <t>2025-04</t>
-        </is>
-      </c>
-      <c r="B45" s="40" t="inlineStr">
-        <is>
-          <t>Paid in Full</t>
-        </is>
-      </c>
-      <c r="C45" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D45" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="E45" s="27" t="n">
-        <v>0</v>
-      </c>
+      <c r="C45" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D45" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E45" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="27" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="25" t="inlineStr">
+      <c r="A46" s="27" t="inlineStr">
         <is>
           <t>2025-05</t>
         </is>
       </c>
       <c r="B46" s="40" t="inlineStr">
         <is>
-          <t>Paid in Full</t>
-        </is>
-      </c>
-      <c r="C46" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D46" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="E46" s="27" t="n">
-        <v>0</v>
+          <t>Paid Late</t>
+        </is>
+      </c>
+      <c r="C46" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D46" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E46" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="27" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-01-29</t>
+        </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="25" t="inlineStr">
+      <c r="A47" s="27" t="inlineStr">
         <is>
           <t>2025-06</t>
         </is>
       </c>
-      <c r="B47" s="38" t="inlineStr">
+      <c r="B47" s="42" t="inlineStr">
         <is>
           <t>Overpayment</t>
         </is>
       </c>
-      <c r="C47" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D47" s="27" t="n">
+      <c r="C47" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D47" s="29" t="n">
         <v>1500</v>
       </c>
       <c r="E47" s="39" t="n">
         <v>-150</v>
       </c>
+      <c r="F47" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="27" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="25" t="inlineStr">
+      <c r="A48" s="27" t="inlineStr">
         <is>
           <t>2025-07</t>
         </is>
       </c>
       <c r="B48" s="40" t="inlineStr">
         <is>
-          <t>Paid in Full</t>
-        </is>
-      </c>
-      <c r="C48" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D48" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="E48" s="27" t="n">
-        <v>0</v>
+          <t>Paid Late</t>
+        </is>
+      </c>
+      <c r="C48" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D48" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E48" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="27" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-07-31</t>
+        </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="25" t="inlineStr">
+      <c r="A49" s="27" t="inlineStr">
         <is>
           <t>2025-08</t>
         </is>
       </c>
       <c r="B49" s="38" t="inlineStr">
         <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="C49" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D49" s="27" t="n">
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="C49" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D49" s="29" t="n">
         <v>1400</v>
       </c>
       <c r="E49" s="39" t="n">
         <v>-50</v>
       </c>
+      <c r="F49" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="27" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2025-08-24</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="25" t="inlineStr">
+      <c r="A50" s="27" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
       </c>
       <c r="B50" s="38" t="inlineStr">
         <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="C50" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D50" s="27" t="n">
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="C50" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D50" s="29" t="n">
         <v>2150</v>
       </c>
       <c r="E50" s="39" t="n">
         <v>-800</v>
       </c>
+      <c r="F50" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="27" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-03-07</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="25" t="inlineStr">
+      <c r="A51" s="27" t="inlineStr">
         <is>
           <t>2025-10</t>
         </is>
       </c>
       <c r="B51" s="38" t="inlineStr">
         <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="C51" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D51" s="27" t="n">
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="C51" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D51" s="29" t="n">
         <v>1550</v>
       </c>
       <c r="E51" s="39" t="n">
         <v>-200</v>
       </c>
+      <c r="F51" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="27" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="25" t="inlineStr">
+      <c r="A52" s="27" t="inlineStr">
         <is>
           <t>2025-11</t>
         </is>
       </c>
       <c r="B52" s="38" t="inlineStr">
         <is>
-          <t>Overpayment</t>
-        </is>
-      </c>
-      <c r="C52" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D52" s="27" t="n">
+          <t>Overpayment / Paid Late</t>
+        </is>
+      </c>
+      <c r="C52" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D52" s="29" t="n">
         <v>1400</v>
       </c>
       <c r="E52" s="39" t="n">
         <v>-50</v>
       </c>
+      <c r="F52" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="27" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-01-07</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="25" t="inlineStr">
+      <c r="A53" s="27" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
       </c>
       <c r="B53" s="40" t="inlineStr">
         <is>
-          <t>Paid in Full</t>
-        </is>
-      </c>
-      <c r="C53" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D53" s="27" t="n">
-        <v>1350</v>
-      </c>
-      <c r="E53" s="27" t="n">
-        <v>0</v>
+          <t>Paid Late</t>
+        </is>
+      </c>
+      <c r="C53" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D53" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E53" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="27" t="inlineStr">
+        <is>
+          <t>Paid after due date on 2026-03-07</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance Rent Management with Monthly Override Features
- Updated MonthlyOverrideDialog to include rental period, default due day, and various overrides (monthly exceptions, due day overrides, late status overrides) for tenants.
- Improved process_monthly_override method to handle new override options, including applying rent and due day overrides.
- Added detailed debug logging for monthly override actions.
- Modified success messages to reflect changes in overrides applied or removed.
- Introduced a new Excel file (Kamden_rent_export.xlsx) for rent tracking.
- Created unit tests for RentTracker to validate due date overrides and late status handling, ensuring correct behavior for various scenarios.
</commit_message>
<xml_diff>
--- a/Financial Manager/resources/Maria(Current)_rent_export.xlsx
+++ b/Financial Manager/resources/Maria(Current)_rent_export.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Main'!$A$1:$H$77</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'2026'!$A$1:$H$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Main'!$A$1:$H$79</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'2026'!$A$1:$H$41</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'2025'!$A$1:$H$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -198,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -300,6 +300,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -673,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -689,7 +692,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Report Generated: 2026-05-22 20:42:57</t>
+          <t>Report Generated: 2026-06-04 22:01:18</t>
         </is>
       </c>
     </row>
@@ -810,7 +813,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>May 2026</t>
+          <t>June 2026</t>
         </is>
       </c>
     </row>
@@ -853,7 +856,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>1600</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="20">
@@ -883,7 +886,7 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>1600</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="24">
@@ -2319,83 +2322,88 @@
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="10" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B67" s="11" t="n">
+        <v>750</v>
+      </c>
+      <c r="C67" s="12" t="inlineStr">
+        <is>
+          <t>Zelle</t>
+        </is>
+      </c>
+      <c r="D67" s="15" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="E67" s="25" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
+        </is>
+      </c>
+      <c r="F67" s="26" t="inlineStr">
+        <is>
+          <t>$600.00 remaining | Late and still owes $600.00</t>
+        </is>
+      </c>
+      <c r="G67" s="11" t="inlineStr"/>
+      <c r="H67" s="12" t="inlineStr">
+        <is>
+          <t>Late and still owes $600.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
         <is>
           <t>MONTHLY BALANCE SUMMARY (Filtered)</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="9" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="9" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B69" s="9" t="inlineStr">
+      <c r="B70" s="9" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C69" s="9" t="inlineStr">
+      <c r="C70" s="9" t="inlineStr">
         <is>
           <t>Rent Due</t>
         </is>
       </c>
-      <c r="D69" s="9" t="inlineStr">
+      <c r="D70" s="9" t="inlineStr">
         <is>
           <t>Total Paid</t>
         </is>
       </c>
-      <c r="E69" s="9" t="inlineStr">
+      <c r="E70" s="9" t="inlineStr">
         <is>
           <t>Balance</t>
         </is>
       </c>
-      <c r="F69" s="9" t="inlineStr">
+      <c r="F70" s="9" t="inlineStr">
         <is>
           <t>Late Fees</t>
         </is>
       </c>
-      <c r="G69" s="9" t="inlineStr">
+      <c r="G70" s="9" t="inlineStr">
         <is>
           <t>Late Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="27" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B70" s="28" t="inlineStr">
-        <is>
-          <t>Delinquent</t>
-        </is>
-      </c>
-      <c r="C70" s="29" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D70" s="29" t="n">
-        <v>1100</v>
-      </c>
-      <c r="E70" s="30" t="n">
-        <v>250</v>
-      </c>
-      <c r="F70" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G70" s="27" t="inlineStr">
-        <is>
-          <t>Late and still owes $250.00</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="27" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B71" s="28" t="inlineStr">
@@ -2407,54 +2415,58 @@
         <v>1350</v>
       </c>
       <c r="D71" s="29" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="E71" s="30" t="n">
-        <v>1350</v>
+        <v>250</v>
       </c>
       <c r="F71" s="29" t="n">
         <v>0</v>
       </c>
       <c r="G71" s="27" t="inlineStr">
         <is>
-          <t>Late and still owes $1350.00</t>
+          <t>Late and still owes $250.00</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="27" t="inlineStr">
         <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B72" s="31" t="inlineStr">
-        <is>
-          <t>Due Soon</t>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B72" s="28" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
         </is>
       </c>
       <c r="C72" s="29" t="n">
         <v>1350</v>
       </c>
       <c r="D72" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E72" s="32" t="n">
-        <v>1350</v>
+        <v>750</v>
+      </c>
+      <c r="E72" s="30" t="n">
+        <v>600</v>
       </c>
       <c r="F72" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="G72" s="27" t="inlineStr"/>
+      <c r="G72" s="27" t="inlineStr">
+        <is>
+          <t>Late and still owes $600.00</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="27" t="inlineStr">
         <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B73" s="33" t="inlineStr">
-        <is>
-          <t>Not Due</t>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B73" s="28" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
         </is>
       </c>
       <c r="C73" s="29" t="n">
@@ -2463,23 +2475,27 @@
       <c r="D73" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="E73" s="34" t="n">
-        <v>0</v>
+      <c r="E73" s="30" t="n">
+        <v>1350</v>
       </c>
       <c r="F73" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="G73" s="27" t="inlineStr"/>
+      <c r="G73" s="27" t="inlineStr">
+        <is>
+          <t>Late and still owes $1350.00</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="27" t="inlineStr">
         <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B74" s="33" t="inlineStr">
-        <is>
-          <t>Not Due</t>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B74" s="31" t="inlineStr">
+        <is>
+          <t>Due Soon</t>
         </is>
       </c>
       <c r="C74" s="29" t="n">
@@ -2488,8 +2504,8 @@
       <c r="D74" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="E74" s="34" t="n">
-        <v>0</v>
+      <c r="E74" s="32" t="n">
+        <v>1350</v>
       </c>
       <c r="F74" s="29" t="n">
         <v>0</v>
@@ -2499,7 +2515,7 @@
     <row r="75">
       <c r="A75" s="27" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B75" s="33" t="inlineStr">
@@ -2524,7 +2540,7 @@
     <row r="76">
       <c r="A76" s="27" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="B76" s="33" t="inlineStr">
@@ -2549,34 +2565,84 @@
     <row r="77">
       <c r="A77" s="27" t="inlineStr">
         <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B77" s="33" t="inlineStr">
+        <is>
+          <t>Not Due</t>
+        </is>
+      </c>
+      <c r="C77" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D77" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="27" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="27" t="inlineStr">
+        <is>
           <t>2026-11</t>
         </is>
       </c>
-      <c r="B77" s="33" t="inlineStr">
+      <c r="B78" s="33" t="inlineStr">
         <is>
           <t>Not Due</t>
         </is>
       </c>
-      <c r="C77" s="29" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D77" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E77" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F77" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G77" s="27" t="inlineStr"/>
+      <c r="C78" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D78" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="27" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="27" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B79" s="33" t="inlineStr">
+        <is>
+          <t>Not Due</t>
+        </is>
+      </c>
+      <c r="C79" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D79" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="27" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A69:H69"/>
     <mergeCell ref="A24:H24"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A68:H68"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -2592,7 +2658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2608,7 +2674,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Report Generated: 2026-05-22 20:42:58 | Year: 2026 (Filtered by Payment Month)</t>
+          <t>Report Generated: 2026-06-04 22:01:18 | Year: 2026 (Filtered by Payment Month)</t>
         </is>
       </c>
     </row>
@@ -3031,120 +3097,125 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="10" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>750</v>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Zelle</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="E21" s="25" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
+        </is>
+      </c>
+      <c r="F21" s="26" t="inlineStr">
+        <is>
+          <t>$600.00 remaining | Late and still owes $600.00</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr"/>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>Late and still owes $600.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>YEAR SUMMARY - 2026 (Tax Purposes)</t>
         </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Total Actual Payments</t>
-        </is>
-      </c>
-      <c r="B23" s="35" t="n">
-        <v>4850</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Total Rent Due</t>
-        </is>
-      </c>
-      <c r="B24" s="36" t="n">
-        <v>16200</v>
+          <t>Total Actual Payments</t>
+        </is>
+      </c>
+      <c r="B24" s="35" t="n">
+        <v>5600</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
+          <t>Total Rent Due</t>
+        </is>
+      </c>
+      <c r="B25" s="36" t="n">
+        <v>16200</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
           <t>Net Difference</t>
         </is>
       </c>
-      <c r="B25" s="37" t="n">
-        <v>-11350</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="B26" s="37" t="n">
+        <v>-10600</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>MONTHLY BALANCE SUMMARY - 2026</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t>Rent Due</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>Total Paid</t>
         </is>
       </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="E29" s="9" t="inlineStr">
         <is>
           <t>Balance</t>
         </is>
       </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>Late Fees</t>
         </is>
       </c>
-      <c r="G28" s="9" t="inlineStr">
+      <c r="G29" s="9" t="inlineStr">
         <is>
           <t>Late Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="27" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B29" s="38" t="inlineStr">
-        <is>
-          <t>Overpayment / Paid Late</t>
-        </is>
-      </c>
-      <c r="C29" s="29" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D29" s="29" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E29" s="39" t="n">
-        <v>-150</v>
-      </c>
-      <c r="F29" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="27" t="inlineStr">
-        <is>
-          <t>Paid after due date on 2026-02-04</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B30" s="38" t="inlineStr">
@@ -3156,141 +3227,145 @@
         <v>1350</v>
       </c>
       <c r="D30" s="29" t="n">
-        <v>1550</v>
+        <v>1500</v>
       </c>
       <c r="E30" s="39" t="n">
-        <v>-200</v>
+        <v>-150</v>
       </c>
       <c r="F30" s="29" t="n">
         <v>0</v>
       </c>
       <c r="G30" s="27" t="inlineStr">
         <is>
-          <t>Paid after due date on 2026-04-01</t>
+          <t>Paid after due date on 2026-02-04</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B31" s="28" t="inlineStr">
-        <is>
-          <t>Delinquent</t>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B31" s="38" t="inlineStr">
+        <is>
+          <t>Overpayment / Paid Late</t>
         </is>
       </c>
       <c r="C31" s="29" t="n">
         <v>1350</v>
       </c>
       <c r="D31" s="29" t="n">
-        <v>1100</v>
-      </c>
-      <c r="E31" s="30" t="n">
-        <v>250</v>
+        <v>1550</v>
+      </c>
+      <c r="E31" s="39" t="n">
+        <v>-200</v>
       </c>
       <c r="F31" s="29" t="n">
         <v>0</v>
       </c>
       <c r="G31" s="27" t="inlineStr">
         <is>
-          <t>Late and still owes $250.00</t>
+          <t>Paid after due date on 2026-04-01</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B32" s="40" t="inlineStr">
-        <is>
-          <t>Paid Late</t>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B32" s="28" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
         </is>
       </c>
       <c r="C32" s="29" t="n">
         <v>1350</v>
       </c>
       <c r="D32" s="29" t="n">
-        <v>1350</v>
-      </c>
-      <c r="E32" s="29" t="n">
-        <v>0</v>
+        <v>1100</v>
+      </c>
+      <c r="E32" s="30" t="n">
+        <v>250</v>
       </c>
       <c r="F32" s="29" t="n">
         <v>0</v>
       </c>
       <c r="G32" s="27" t="inlineStr">
         <is>
-          <t>Paid after due date on 2026-05-22</t>
+          <t>Late and still owes $250.00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B33" s="28" t="inlineStr">
-        <is>
-          <t>Delinquent</t>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B33" s="40" t="inlineStr">
+        <is>
+          <t>Paid Late</t>
         </is>
       </c>
       <c r="C33" s="29" t="n">
         <v>1350</v>
       </c>
       <c r="D33" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="30" t="n">
-        <v>1350</v>
+        <v>1350</v>
+      </c>
+      <c r="E33" s="41" t="n">
+        <v>0</v>
       </c>
       <c r="F33" s="29" t="n">
         <v>0</v>
       </c>
       <c r="G33" s="27" t="inlineStr">
         <is>
-          <t>Late and still owes $1350.00</t>
+          <t>Paid after due date on 2026-05-22</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B34" s="31" t="inlineStr">
-        <is>
-          <t>Due Soon</t>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B34" s="28" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
         </is>
       </c>
       <c r="C34" s="29" t="n">
         <v>1350</v>
       </c>
       <c r="D34" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="32" t="n">
-        <v>1350</v>
+        <v>750</v>
+      </c>
+      <c r="E34" s="30" t="n">
+        <v>600</v>
       </c>
       <c r="F34" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="G34" s="27" t="inlineStr"/>
+      <c r="G34" s="27" t="inlineStr">
+        <is>
+          <t>Late and still owes $600.00</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B35" s="33" t="inlineStr">
-        <is>
-          <t>Not Due</t>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B35" s="28" t="inlineStr">
+        <is>
+          <t>Delinquent</t>
         </is>
       </c>
       <c r="C35" s="29" t="n">
@@ -3299,23 +3374,27 @@
       <c r="D35" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="E35" s="34" t="n">
-        <v>0</v>
+      <c r="E35" s="30" t="n">
+        <v>1350</v>
       </c>
       <c r="F35" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="G35" s="27" t="inlineStr"/>
+      <c r="G35" s="27" t="inlineStr">
+        <is>
+          <t>Late and still owes $1350.00</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B36" s="33" t="inlineStr">
-        <is>
-          <t>Not Due</t>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B36" s="31" t="inlineStr">
+        <is>
+          <t>Due Soon</t>
         </is>
       </c>
       <c r="C36" s="29" t="n">
@@ -3324,8 +3403,8 @@
       <c r="D36" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="E36" s="34" t="n">
-        <v>0</v>
+      <c r="E36" s="32" t="n">
+        <v>1350</v>
       </c>
       <c r="F36" s="29" t="n">
         <v>0</v>
@@ -3335,7 +3414,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B37" s="33" t="inlineStr">
@@ -3360,7 +3439,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="B38" s="33" t="inlineStr">
@@ -3385,7 +3464,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>2026-11</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="B39" s="33" t="inlineStr">
@@ -3410,36 +3489,61 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B40" s="33" t="inlineStr">
+        <is>
+          <t>Not Due</t>
+        </is>
+      </c>
+      <c r="C40" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D40" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="27" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="27" t="inlineStr">
+        <is>
           <t>2026-12</t>
         </is>
       </c>
-      <c r="B40" s="33" t="inlineStr">
+      <c r="B41" s="33" t="inlineStr">
         <is>
           <t>Not Due</t>
         </is>
       </c>
-      <c r="C40" s="29" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D40" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" s="27" t="inlineStr"/>
+      <c r="C41" s="29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D41" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="27" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A23:H23"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3469,7 +3573,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Report Generated: 2026-05-22 20:42:58 | Year: 2025 (Filtered by Date Received)</t>
+          <t>Report Generated: 2026-06-04 22:01:19 | Year: 2025 (Filtered by Date Received)</t>
         </is>
       </c>
     </row>
@@ -4397,7 +4501,7 @@
           <t>2025-01</t>
         </is>
       </c>
-      <c r="B42" s="41" t="inlineStr">
+      <c r="B42" s="42" t="inlineStr">
         <is>
           <t>Paid in Full</t>
         </is>
@@ -4408,7 +4512,7 @@
       <c r="D42" s="29" t="n">
         <v>1350</v>
       </c>
-      <c r="E42" s="29" t="n">
+      <c r="E42" s="39" t="n">
         <v>0</v>
       </c>
       <c r="F42" s="29" t="n">
@@ -4422,7 +4526,7 @@
           <t>2025-02</t>
         </is>
       </c>
-      <c r="B43" s="41" t="inlineStr">
+      <c r="B43" s="42" t="inlineStr">
         <is>
           <t>Paid in Full</t>
         </is>
@@ -4433,7 +4537,7 @@
       <c r="D43" s="29" t="n">
         <v>1350</v>
       </c>
-      <c r="E43" s="29" t="n">
+      <c r="E43" s="39" t="n">
         <v>0</v>
       </c>
       <c r="F43" s="29" t="n">
@@ -4458,7 +4562,7 @@
       <c r="D44" s="29" t="n">
         <v>1350</v>
       </c>
-      <c r="E44" s="29" t="n">
+      <c r="E44" s="41" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="29" t="n">
@@ -4476,7 +4580,7 @@
           <t>2025-04</t>
         </is>
       </c>
-      <c r="B45" s="41" t="inlineStr">
+      <c r="B45" s="42" t="inlineStr">
         <is>
           <t>Paid in Full</t>
         </is>
@@ -4487,7 +4591,7 @@
       <c r="D45" s="29" t="n">
         <v>1350</v>
       </c>
-      <c r="E45" s="29" t="n">
+      <c r="E45" s="39" t="n">
         <v>0</v>
       </c>
       <c r="F45" s="29" t="n">
@@ -4512,7 +4616,7 @@
       <c r="D46" s="29" t="n">
         <v>1350</v>
       </c>
-      <c r="E46" s="29" t="n">
+      <c r="E46" s="41" t="n">
         <v>0</v>
       </c>
       <c r="F46" s="29" t="n">
@@ -4530,7 +4634,7 @@
           <t>2025-06</t>
         </is>
       </c>
-      <c r="B47" s="42" t="inlineStr">
+      <c r="B47" s="43" t="inlineStr">
         <is>
           <t>Overpayment</t>
         </is>
@@ -4566,7 +4670,7 @@
       <c r="D48" s="29" t="n">
         <v>1350</v>
       </c>
-      <c r="E48" s="29" t="n">
+      <c r="E48" s="41" t="n">
         <v>0</v>
       </c>
       <c r="F48" s="29" t="n">
@@ -4711,7 +4815,7 @@
       <c r="D53" s="29" t="n">
         <v>1350</v>
       </c>
-      <c r="E53" s="29" t="n">
+      <c r="E53" s="41" t="n">
         <v>0</v>
       </c>
       <c r="F53" s="29" t="n">

</xml_diff>